<commit_message>
Hyderabad FG mismatch: correct three notes per verification advisories
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SVVKmwQKKV189dev92iFna
</commit_message>
<xml_diff>
--- a/reports/Hyderabad-FG-Mismatch-2026-10-29.xlsx
+++ b/reports/Hyderabad-FG-Mismatch-2026-10-29.xlsx
@@ -131,7 +131,7 @@
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
-    <t xml:space="preserve">Plant sheet rows "25.4OD" are matched to the system's CHS 20 NB (the system has no 25.4 OD size; tonnages track closely at every thickness).</t>
+    <t xml:space="preserve">Plant sheet rows "25.4OD" are matched to the system's CHS 20 NB (assumption: the system has no 25.4 OD size and no 20 NB row is on the plant sheet; same thicknesses, system 2-3 MT higher at three of four).</t>
   </si>
   <si>
     <t xml:space="preserve">Thickness 2.8, 2.9, 3.0 and 3.2 of the same size are counted as one size (3.0), as decided on 29-Oct; the "Thickness detail" sheet shows the codes underneath.</t>
@@ -140,13 +140,13 @@
     <t xml:space="preserve">System FG = produced minus invoiced at Hyderabad, per size, never below 0; invoices use up the oldest production first (approved Inventory Snapshot rules S1, S2, S10).</t>
   </si>
   <si>
-    <t xml:space="preserve">Hyderabad has no invoice in the system dated after 26-Oct. Dispatches of 27-28 Oct, if any, are not yet in the figures.</t>
+    <t xml:space="preserve">Hyderabad has no invoice in the system dated after 26-Oct, although the same register upload has 27-28 Oct invoices for NPMD and Tapi. Either Hyderabad billed nothing on 27-28 Oct, or its rows were dropped as an unrecognised warehouse name (the upload banner lists skipped warehouses).</t>
   </si>
   <si>
     <t xml:space="preserve">Production before tracking began (28-Mar-2026) is not in the system, so stock made before then and sold after shows as "billed beyond production".</t>
   </si>
   <si>
-    <t xml:space="preserve">The plant sheet's 55 visible rows add up to 643.432 MT against its Grand Total of 649.586 MT; please check for hidden or filtered rows (6.154 MT).</t>
+    <t xml:space="preserve">The plant sheet's 55 visible rows add up to 643.432 MT against its Grand Total of 649.586 MT; please check for hidden or filtered rows (6.154 MT). The sheet's own Free total (443.339) is also 0.247 MT below Grand Total minus Reserved (443.586).</t>
   </si>
   <si>
     <t xml:space="preserve">Hyderabad FG - sizes where the plant sheet and the system do not match</t>
@@ -305,7 +305,7 @@
     <t xml:space="preserve">80X40X2</t>
   </si>
   <si>
-    <t xml:space="preserve">System higher: check for dispatches not yet invoiced (no Hyderabad invoice in the system after 26-Oct) and stock billed under a neighbouring code.</t>
+    <t xml:space="preserve">System higher: check for Hyderabad dispatches of 27-28 Oct (none invoiced in the system after 26-Oct) and stock billed under a neighbouring code.</t>
   </si>
   <si>
     <t xml:space="preserve">60X40X2.8</t>

</xml_diff>